<commit_message>
Update Excel report with latest test run results
</commit_message>
<xml_diff>
--- a/Selenium_Web_300_Test_Report.xlsx
+++ b/Selenium_Web_300_Test_Report.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>10.22 s</t>
+          <t>10.84 s</t>
         </is>
       </c>
     </row>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="F2" s="17" t="n">
-        <v>2.5626</v>
+        <v>2.639</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:18</t>
+          <t>2026-08-07 09:24:55</t>
         </is>
       </c>
       <c r="H2" s="15" t="inlineStr">
@@ -1001,11 +1001,11 @@
         </is>
       </c>
       <c r="F3" s="17" t="n">
-        <v>0.0053</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
@@ -1041,11 +1041,11 @@
         </is>
       </c>
       <c r="F4" s="17" t="n">
-        <v>0.0332</v>
+        <v>0.0304</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
@@ -1081,11 +1081,11 @@
         </is>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.0245</v>
+        <v>0.0261</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -1121,11 +1121,11 @@
         </is>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.0274</v>
+        <v>0.025</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -1161,11 +1161,11 @@
         </is>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0.0468</v>
+        <v>0.0473</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="F8" s="17" t="n">
-        <v>0.0106</v>
+        <v>0.014</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -1241,11 +1241,11 @@
         </is>
       </c>
       <c r="F9" s="17" t="n">
-        <v>0.056</v>
+        <v>0.0468</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:57</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -1281,11 +1281,11 @@
         </is>
       </c>
       <c r="F10" s="17" t="n">
-        <v>0.05</v>
+        <v>0.0501</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
@@ -1321,11 +1321,11 @@
         </is>
       </c>
       <c r="F11" s="17" t="n">
-        <v>0.0295</v>
+        <v>0.0222</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H24" s="15" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H26" s="15" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H27" s="15" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H28" s="15" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H29" s="15" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H30" s="15" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H31" s="15" t="inlineStr">
@@ -2161,11 +2161,11 @@
         </is>
       </c>
       <c r="F32" s="17" t="n">
-        <v>1.9281</v>
+        <v>1.8649</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:21</t>
+          <t>2026-08-07 09:24:58</t>
         </is>
       </c>
       <c r="H32" s="15" t="inlineStr">
@@ -2204,11 +2204,11 @@
         </is>
       </c>
       <c r="F33" s="17" t="n">
-        <v>0.0162</v>
+        <v>0.0167</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:23</t>
+          <t>2026-08-07 09:24:59</t>
         </is>
       </c>
       <c r="H33" s="15" t="inlineStr">
@@ -2244,11 +2244,11 @@
         </is>
       </c>
       <c r="F34" s="17" t="n">
-        <v>0.0137</v>
+        <v>0.0143</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:23</t>
+          <t>2026-08-07 09:24:59</t>
         </is>
       </c>
       <c r="H34" s="15" t="inlineStr">
@@ -2284,11 +2284,11 @@
         </is>
       </c>
       <c r="F35" s="17" t="n">
-        <v>0.0129</v>
+        <v>0.0147</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:23</t>
+          <t>2026-08-07 09:24:59</t>
         </is>
       </c>
       <c r="H35" s="15" t="inlineStr">
@@ -2324,11 +2324,11 @@
         </is>
       </c>
       <c r="F36" s="17" t="n">
-        <v>0.4251</v>
+        <v>0.4902</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:23</t>
+          <t>2026-08-07 09:24:59</t>
         </is>
       </c>
       <c r="H36" s="15" t="inlineStr">
@@ -2367,11 +2367,11 @@
         </is>
       </c>
       <c r="F37" s="17" t="n">
-        <v>0.0274</v>
+        <v>0.0304</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:23</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H37" s="15" t="inlineStr">
@@ -2407,11 +2407,11 @@
         </is>
       </c>
       <c r="F38" s="17" t="n">
-        <v>0.0275</v>
+        <v>0.0283</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:23</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H38" s="15" t="inlineStr">
@@ -2447,11 +2447,11 @@
         </is>
       </c>
       <c r="F39" s="17" t="n">
-        <v>0.0265</v>
+        <v>0.0266</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H39" s="15" t="inlineStr">
@@ -2487,11 +2487,11 @@
         </is>
       </c>
       <c r="F40" s="17" t="n">
-        <v>0.0239</v>
+        <v>0.0268</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H40" s="15" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H41" s="15" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H42" s="15" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H43" s="15" t="inlineStr">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H44" s="15" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H46" s="15" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H47" s="15" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H48" s="15" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H49" s="15" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H50" s="15" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H51" s="15" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H52" s="15" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H53" s="15" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H54" s="15" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H55" s="15" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H56" s="15" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H57" s="15" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H58" s="15" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H59" s="15" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H60" s="15" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H61" s="15" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H62" s="15" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H63" s="15" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H64" s="15" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H66" s="15" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H67" s="15" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="G68" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H68" s="15" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H69" s="15" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="G70" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H70" s="15" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="G71" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H71" s="15" t="inlineStr">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="G72" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H72" s="15" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="G73" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H73" s="15" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="G74" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H74" s="15" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H75" s="15" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="G77" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H77" s="15" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G78" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H78" s="15" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H79" s="15" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="G80" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H80" s="15" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="G81" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H81" s="15" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="G82" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H82" s="15" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="G83" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H83" s="15" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H84" s="15" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H85" s="15" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H86" s="15" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="G87" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H87" s="15" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G88" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H88" s="15" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G89" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H89" s="15" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="G90" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H90" s="15" t="inlineStr">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="G91" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H91" s="15" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="G92" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H92" s="15" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G93" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H93" s="15" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="G94" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H94" s="15" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="G95" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H95" s="15" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="G96" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H96" s="15" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="G97" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H97" s="15" t="inlineStr">
@@ -4811,7 +4811,7 @@
       </c>
       <c r="G98" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H98" s="15" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="G99" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H99" s="15" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="G100" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H100" s="15" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="G101" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H101" s="15" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="G102" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H102" s="15" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="G103" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H103" s="15" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="G104" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H104" s="15" t="inlineStr">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="G105" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H105" s="15" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="G106" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H106" s="15" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="G107" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H107" s="15" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G108" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H108" s="15" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="G109" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H109" s="15" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G110" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H110" s="15" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="G111" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H111" s="15" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="G112" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H112" s="15" t="inlineStr">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="G113" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H113" s="15" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="G114" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H114" s="15" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="G115" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H115" s="15" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="G116" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H116" s="15" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="G117" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H117" s="15" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G118" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H118" s="15" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="G119" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H119" s="15" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="G120" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H120" s="15" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G121" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H121" s="15" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="G122" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H122" s="15" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="G123" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H123" s="15" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G124" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H124" s="15" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="G125" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H125" s="15" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="G126" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H126" s="15" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="G127" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H127" s="15" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="G128" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H128" s="15" t="inlineStr">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="G129" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H129" s="15" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="G130" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H130" s="15" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="G131" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H131" s="15" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G132" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H132" s="15" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G133" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H133" s="15" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="G134" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H134" s="15" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="G135" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H135" s="15" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="G136" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H136" s="15" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="G137" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H137" s="15" t="inlineStr">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="G138" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H138" s="15" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="G139" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H139" s="15" t="inlineStr">
@@ -6487,11 +6487,11 @@
         </is>
       </c>
       <c r="F140" s="17" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G140" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H140" s="15" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="G141" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H141" s="15" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="G142" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H142" s="15" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G143" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H143" s="15" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="G144" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H144" s="15" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="G145" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H145" s="15" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="G146" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H146" s="15" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="G147" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H147" s="15" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G148" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H148" s="15" t="inlineStr">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="G149" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H149" s="15" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="G150" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H150" s="15" t="inlineStr">
@@ -6931,7 +6931,7 @@
       </c>
       <c r="G151" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H151" s="15" t="inlineStr">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="G152" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H152" s="15" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="G153" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H153" s="15" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="G154" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H154" s="15" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="G155" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H155" s="15" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="G156" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H156" s="15" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G157" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H157" s="15" t="inlineStr">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G158" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H158" s="15" t="inlineStr">
@@ -7251,7 +7251,7 @@
       </c>
       <c r="G159" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H159" s="15" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="G160" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H160" s="15" t="inlineStr">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="G161" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H161" s="15" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="G162" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H162" s="15" t="inlineStr">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="G163" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H163" s="15" t="inlineStr">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="G164" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H164" s="15" t="inlineStr">
@@ -7487,11 +7487,11 @@
         </is>
       </c>
       <c r="F165" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G165" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H165" s="15" t="inlineStr">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="G166" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H166" s="15" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="G167" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H167" s="15" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G168" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H168" s="15" t="inlineStr">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="G169" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H169" s="15" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="G170" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H170" s="15" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="G171" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H171" s="15" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="G172" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H172" s="15" t="inlineStr">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="G173" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H173" s="15" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="G174" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H174" s="15" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H175" s="15" t="inlineStr">
@@ -7931,7 +7931,7 @@
       </c>
       <c r="G176" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H176" s="15" t="inlineStr">
@@ -7971,7 +7971,7 @@
       </c>
       <c r="G177" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H177" s="15" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G178" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H178" s="15" t="inlineStr">
@@ -8051,7 +8051,7 @@
       </c>
       <c r="G179" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H179" s="15" t="inlineStr">
@@ -8091,7 +8091,7 @@
       </c>
       <c r="G180" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H180" s="15" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="G181" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H181" s="15" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="G182" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H182" s="15" t="inlineStr">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="G183" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H183" s="15" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="G184" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H184" s="15" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="G185" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H185" s="15" t="inlineStr">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="G186" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H186" s="15" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="G187" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H187" s="15" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="G188" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H188" s="15" t="inlineStr">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="G189" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H189" s="15" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="G190" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H190" s="15" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="G191" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H191" s="15" t="inlineStr">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="G192" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H192" s="15" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="G193" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H193" s="15" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="G194" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H194" s="15" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G195" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H195" s="15" t="inlineStr">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="G196" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H196" s="15" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="G197" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H197" s="15" t="inlineStr">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G198" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H198" s="15" t="inlineStr">
@@ -8851,7 +8851,7 @@
       </c>
       <c r="G199" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H199" s="15" t="inlineStr">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="G200" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H200" s="15" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="G201" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H201" s="15" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="G202" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H202" s="15" t="inlineStr">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G203" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H203" s="15" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="G204" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H204" s="15" t="inlineStr">
@@ -9091,7 +9091,7 @@
       </c>
       <c r="G205" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H205" s="15" t="inlineStr">
@@ -9131,7 +9131,7 @@
       </c>
       <c r="G206" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H206" s="15" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="G207" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H207" s="15" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G208" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H208" s="15" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="G209" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H209" s="15" t="inlineStr">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="G210" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H210" s="15" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="G211" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H211" s="15" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="G212" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H212" s="15" t="inlineStr">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="G213" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H213" s="15" t="inlineStr">
@@ -9451,7 +9451,7 @@
       </c>
       <c r="G214" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H214" s="15" t="inlineStr">
@@ -9491,7 +9491,7 @@
       </c>
       <c r="G215" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H215" s="15" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="G216" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H216" s="15" t="inlineStr">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="G217" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H217" s="15" t="inlineStr">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G218" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H218" s="15" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="G219" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H219" s="15" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="G220" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H220" s="15" t="inlineStr">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="G221" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H221" s="15" t="inlineStr">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="G222" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H222" s="15" t="inlineStr">
@@ -9811,7 +9811,7 @@
       </c>
       <c r="G223" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H223" s="15" t="inlineStr">
@@ -9851,7 +9851,7 @@
       </c>
       <c r="G224" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H224" s="15" t="inlineStr">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="G225" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H225" s="15" t="inlineStr">
@@ -9931,7 +9931,7 @@
       </c>
       <c r="G226" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H226" s="15" t="inlineStr">
@@ -9971,7 +9971,7 @@
       </c>
       <c r="G227" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H227" s="15" t="inlineStr">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="G228" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H228" s="15" t="inlineStr">
@@ -10051,7 +10051,7 @@
       </c>
       <c r="G229" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H229" s="15" t="inlineStr">
@@ -10091,7 +10091,7 @@
       </c>
       <c r="G230" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H230" s="15" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="G231" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H231" s="15" t="inlineStr">
@@ -10171,7 +10171,7 @@
       </c>
       <c r="G232" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H232" s="15" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="G233" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H233" s="15" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="G234" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H234" s="15" t="inlineStr">
@@ -10291,7 +10291,7 @@
       </c>
       <c r="G235" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H235" s="15" t="inlineStr">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="G236" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H236" s="15" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="G237" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H237" s="15" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="G238" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H238" s="15" t="inlineStr">
@@ -10451,7 +10451,7 @@
       </c>
       <c r="G239" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H239" s="15" t="inlineStr">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="G240" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H240" s="15" t="inlineStr">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="G241" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H241" s="15" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="G242" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H242" s="15" t="inlineStr">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="G243" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H243" s="15" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="G244" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H244" s="15" t="inlineStr">
@@ -10691,7 +10691,7 @@
       </c>
       <c r="G245" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H245" s="15" t="inlineStr">
@@ -10731,7 +10731,7 @@
       </c>
       <c r="G246" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H246" s="15" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="G247" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H247" s="15" t="inlineStr">
@@ -10811,7 +10811,7 @@
       </c>
       <c r="G248" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H248" s="15" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="G249" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H249" s="15" t="inlineStr">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="G250" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H250" s="15" t="inlineStr">
@@ -10931,7 +10931,7 @@
       </c>
       <c r="G251" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H251" s="15" t="inlineStr">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="G252" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H252" s="15" t="inlineStr">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="G253" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H253" s="15" t="inlineStr">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="G254" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H254" s="15" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="G255" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H255" s="15" t="inlineStr">
@@ -11131,7 +11131,7 @@
       </c>
       <c r="G256" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H256" s="15" t="inlineStr">
@@ -11171,7 +11171,7 @@
       </c>
       <c r="G257" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H257" s="15" t="inlineStr">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="G258" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H258" s="15" t="inlineStr">
@@ -11251,7 +11251,7 @@
       </c>
       <c r="G259" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H259" s="15" t="inlineStr">
@@ -11291,7 +11291,7 @@
       </c>
       <c r="G260" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H260" s="15" t="inlineStr">
@@ -11331,7 +11331,7 @@
       </c>
       <c r="G261" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H261" s="15" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="G262" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H262" s="15" t="inlineStr">
@@ -11407,11 +11407,11 @@
         </is>
       </c>
       <c r="F263" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G263" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H263" s="15" t="inlineStr">
@@ -11451,7 +11451,7 @@
       </c>
       <c r="G264" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H264" s="15" t="inlineStr">
@@ -11491,7 +11491,7 @@
       </c>
       <c r="G265" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H265" s="15" t="inlineStr">
@@ -11531,7 +11531,7 @@
       </c>
       <c r="G266" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H266" s="15" t="inlineStr">
@@ -11571,7 +11571,7 @@
       </c>
       <c r="G267" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H267" s="15" t="inlineStr">
@@ -11611,7 +11611,7 @@
       </c>
       <c r="G268" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H268" s="15" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="G269" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H269" s="15" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="G270" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H270" s="15" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="G271" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H271" s="15" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="G272" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H272" s="15" t="inlineStr">
@@ -11811,7 +11811,7 @@
       </c>
       <c r="G273" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H273" s="15" t="inlineStr">
@@ -11851,7 +11851,7 @@
       </c>
       <c r="G274" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H274" s="15" t="inlineStr">
@@ -11891,7 +11891,7 @@
       </c>
       <c r="G275" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H275" s="15" t="inlineStr">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="G276" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H276" s="15" t="inlineStr">
@@ -11971,7 +11971,7 @@
       </c>
       <c r="G277" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H277" s="15" t="inlineStr">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="G278" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H278" s="15" t="inlineStr">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="G279" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H279" s="15" t="inlineStr">
@@ -12091,7 +12091,7 @@
       </c>
       <c r="G280" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H280" s="15" t="inlineStr">
@@ -12131,7 +12131,7 @@
       </c>
       <c r="G281" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H281" s="15" t="inlineStr">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="G282" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H282" s="15" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="G283" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H283" s="15" t="inlineStr">
@@ -12251,7 +12251,7 @@
       </c>
       <c r="G284" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H284" s="15" t="inlineStr">
@@ -12291,7 +12291,7 @@
       </c>
       <c r="G285" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H285" s="15" t="inlineStr">
@@ -12331,7 +12331,7 @@
       </c>
       <c r="G286" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H286" s="15" t="inlineStr">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="G287" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H287" s="15" t="inlineStr">
@@ -12411,7 +12411,7 @@
       </c>
       <c r="G288" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H288" s="15" t="inlineStr">
@@ -12451,7 +12451,7 @@
       </c>
       <c r="G289" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H289" s="15" t="inlineStr">
@@ -12491,7 +12491,7 @@
       </c>
       <c r="G290" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H290" s="15" t="inlineStr">
@@ -12531,7 +12531,7 @@
       </c>
       <c r="G291" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H291" s="15" t="inlineStr">
@@ -12571,7 +12571,7 @@
       </c>
       <c r="G292" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H292" s="15" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="G293" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H293" s="15" t="inlineStr">
@@ -12651,7 +12651,7 @@
       </c>
       <c r="G294" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H294" s="15" t="inlineStr">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="G295" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H295" s="15" t="inlineStr">
@@ -12731,7 +12731,7 @@
       </c>
       <c r="G296" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H296" s="15" t="inlineStr">
@@ -12771,7 +12771,7 @@
       </c>
       <c r="G297" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H297" s="15" t="inlineStr">
@@ -12811,7 +12811,7 @@
       </c>
       <c r="G298" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H298" s="15" t="inlineStr">
@@ -12851,7 +12851,7 @@
       </c>
       <c r="G299" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H299" s="15" t="inlineStr">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="G300" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H300" s="15" t="inlineStr">
@@ -12931,7 +12931,7 @@
       </c>
       <c r="G301" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:10:24</t>
+          <t>2026-08-07 09:25:00</t>
         </is>
       </c>
       <c r="H301" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fix blank screen issue on GitHub Pages: add HashRouter, Firebase env fallbacks, and 404 fallback page
</commit_message>
<xml_diff>
--- a/Selenium_Web_300_Test_Report.xlsx
+++ b/Selenium_Web_300_Test_Report.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>10.84 s</t>
+          <t>17.07 s</t>
         </is>
       </c>
     </row>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="F2" s="17" t="n">
-        <v>2.639</v>
+        <v>2.5215</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:55</t>
+          <t>2026-08-07 11:10:30</t>
         </is>
       </c>
       <c r="H2" s="15" t="inlineStr">
@@ -970,7 +970,7 @@
           <t>Verified with condition logic: Message: unknown error: net::ERR_CONNECTION_REFUSED
   (Session info: chrome=150.0.7871.187)
 Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff70bc10d2</t>
+	chromedriver!GetHandleVerifier [0x7ff7d58d0d2</t>
         </is>
       </c>
     </row>
@@ -1001,11 +1001,11 @@
         </is>
       </c>
       <c r="F3" s="17" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0339</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
@@ -1041,11 +1041,11 @@
         </is>
       </c>
       <c r="F4" s="17" t="n">
-        <v>0.0304</v>
+        <v>0.1426</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
@@ -1081,11 +1081,11 @@
         </is>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.0261</v>
+        <v>0.1181</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -1121,11 +1121,11 @@
         </is>
       </c>
       <c r="F6" s="17" t="n">
-        <v>0.025</v>
+        <v>0.0955</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -1161,11 +1161,11 @@
         </is>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0.0473</v>
+        <v>0.1625</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="F8" s="17" t="n">
-        <v>0.014</v>
+        <v>0.0471</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -1241,11 +1241,11 @@
         </is>
       </c>
       <c r="F9" s="17" t="n">
-        <v>0.0468</v>
+        <v>0.2001</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:57</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -1281,11 +1281,11 @@
         </is>
       </c>
       <c r="F10" s="17" t="n">
-        <v>0.0501</v>
+        <v>0.1858</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:33</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
@@ -1321,11 +1321,11 @@
         </is>
       </c>
       <c r="F11" s="17" t="n">
-        <v>0.0222</v>
+        <v>0.0978</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H24" s="15" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H26" s="15" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H27" s="15" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H28" s="15" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H29" s="15" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H30" s="15" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H31" s="15" t="inlineStr">
@@ -2161,11 +2161,11 @@
         </is>
       </c>
       <c r="F32" s="17" t="n">
-        <v>1.8649</v>
+        <v>2.4829</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:58</t>
+          <t>2026-08-07 11:10:34</t>
         </is>
       </c>
       <c r="H32" s="15" t="inlineStr">
@@ -2173,7 +2173,7 @@
           <t>Verified with condition logic: Message: unknown error: net::ERR_CONNECTION_REFUSED
   (Session info: chrome=150.0.7871.187)
 Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff70bc10d2</t>
+	chromedriver!GetHandleVerifier [0x7ff7d58d0d2</t>
         </is>
       </c>
     </row>
@@ -2204,11 +2204,11 @@
         </is>
       </c>
       <c r="F33" s="17" t="n">
-        <v>0.0167</v>
+        <v>0.0704</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:59</t>
+          <t>2026-08-07 11:10:36</t>
         </is>
       </c>
       <c r="H33" s="15" t="inlineStr">
@@ -2244,11 +2244,11 @@
         </is>
       </c>
       <c r="F34" s="17" t="n">
-        <v>0.0143</v>
+        <v>0.0689</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:59</t>
+          <t>2026-08-07 11:10:36</t>
         </is>
       </c>
       <c r="H34" s="15" t="inlineStr">
@@ -2284,11 +2284,11 @@
         </is>
       </c>
       <c r="F35" s="17" t="n">
-        <v>0.0147</v>
+        <v>0.0634</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:59</t>
+          <t>2026-08-07 11:10:36</t>
         </is>
       </c>
       <c r="H35" s="15" t="inlineStr">
@@ -2324,11 +2324,11 @@
         </is>
       </c>
       <c r="F36" s="17" t="n">
-        <v>0.4902</v>
+        <v>2.4819</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:24:59</t>
+          <t>2026-08-07 11:10:36</t>
         </is>
       </c>
       <c r="H36" s="15" t="inlineStr">
@@ -2336,7 +2336,7 @@
           <t>Verified with condition logic: Message: unknown error: net::ERR_CONNECTION_REFUSED
   (Session info: chrome=150.0.7871.187)
 Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff70bc10d2</t>
+	chromedriver!GetHandleVerifier [0x7ff7d58d0d2</t>
         </is>
       </c>
     </row>
@@ -2367,11 +2367,11 @@
         </is>
       </c>
       <c r="F37" s="17" t="n">
-        <v>0.0304</v>
+        <v>0.1355</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H37" s="15" t="inlineStr">
@@ -2407,11 +2407,11 @@
         </is>
       </c>
       <c r="F38" s="17" t="n">
-        <v>0.0283</v>
+        <v>0.1129</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H38" s="15" t="inlineStr">
@@ -2447,11 +2447,11 @@
         </is>
       </c>
       <c r="F39" s="17" t="n">
-        <v>0.0266</v>
+        <v>0.132</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H39" s="15" t="inlineStr">
@@ -2487,11 +2487,11 @@
         </is>
       </c>
       <c r="F40" s="17" t="n">
-        <v>0.0268</v>
+        <v>0.109</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H40" s="15" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H41" s="15" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H42" s="15" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H43" s="15" t="inlineStr">
@@ -2647,11 +2647,11 @@
         </is>
       </c>
       <c r="F44" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H44" s="15" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H46" s="15" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H47" s="15" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H48" s="15" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H49" s="15" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H50" s="15" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H51" s="15" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H52" s="15" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H53" s="15" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H54" s="15" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H55" s="15" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H56" s="15" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H57" s="15" t="inlineStr">
@@ -3207,11 +3207,11 @@
         </is>
       </c>
       <c r="F58" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H58" s="15" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H59" s="15" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H60" s="15" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H61" s="15" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H62" s="15" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H63" s="15" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H64" s="15" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H66" s="15" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H67" s="15" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="G68" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H68" s="15" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H69" s="15" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="G70" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H70" s="15" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="G71" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H71" s="15" t="inlineStr">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="G72" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H72" s="15" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="G73" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H73" s="15" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="G74" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H74" s="15" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H75" s="15" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="G77" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H77" s="15" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G78" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H78" s="15" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H79" s="15" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="G80" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H80" s="15" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="G81" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H81" s="15" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="G82" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H82" s="15" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="G83" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H83" s="15" t="inlineStr">
@@ -4247,11 +4247,11 @@
         </is>
       </c>
       <c r="F84" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H84" s="15" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H85" s="15" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H86" s="15" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="G87" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H87" s="15" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G88" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H88" s="15" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G89" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H89" s="15" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="G90" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H90" s="15" t="inlineStr">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="G91" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H91" s="15" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="G92" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H92" s="15" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G93" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H93" s="15" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="G94" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H94" s="15" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="G95" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H95" s="15" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="G96" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H96" s="15" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="G97" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H97" s="15" t="inlineStr">
@@ -4811,7 +4811,7 @@
       </c>
       <c r="G98" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H98" s="15" t="inlineStr">
@@ -4847,11 +4847,11 @@
         </is>
       </c>
       <c r="F99" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G99" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H99" s="15" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="G100" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H100" s="15" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="G101" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H101" s="15" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="G102" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H102" s="15" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="G103" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H103" s="15" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="G104" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H104" s="15" t="inlineStr">
@@ -5087,11 +5087,11 @@
         </is>
       </c>
       <c r="F105" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G105" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H105" s="15" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="G106" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H106" s="15" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="G107" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H107" s="15" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G108" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H108" s="15" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="G109" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H109" s="15" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G110" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H110" s="15" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="G111" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H111" s="15" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="G112" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H112" s="15" t="inlineStr">
@@ -5407,11 +5407,11 @@
         </is>
       </c>
       <c r="F113" s="17" t="n">
-        <v>0</v>
+        <v>0.0009</v>
       </c>
       <c r="G113" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H113" s="15" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="G114" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H114" s="15" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="G115" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H115" s="15" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="G116" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H116" s="15" t="inlineStr">
@@ -5567,11 +5567,11 @@
         </is>
       </c>
       <c r="F117" s="17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G117" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H117" s="15" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G118" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H118" s="15" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="G119" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H119" s="15" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="G120" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H120" s="15" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G121" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H121" s="15" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="G122" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H122" s="15" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="G123" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H123" s="15" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G124" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H124" s="15" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="G125" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H125" s="15" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="G126" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H126" s="15" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="G127" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H127" s="15" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="G128" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H128" s="15" t="inlineStr">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="G129" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H129" s="15" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="G130" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H130" s="15" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="G131" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H131" s="15" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G132" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H132" s="15" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G133" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H133" s="15" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="G134" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H134" s="15" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="G135" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H135" s="15" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="G136" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H136" s="15" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="G137" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H137" s="15" t="inlineStr">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="G138" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H138" s="15" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="G139" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H139" s="15" t="inlineStr">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="G140" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H140" s="15" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="G141" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H141" s="15" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="G142" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H142" s="15" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G143" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H143" s="15" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="G144" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H144" s="15" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="G145" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H145" s="15" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="G146" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H146" s="15" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="G147" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H147" s="15" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G148" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H148" s="15" t="inlineStr">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="G149" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H149" s="15" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="G150" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H150" s="15" t="inlineStr">
@@ -6931,7 +6931,7 @@
       </c>
       <c r="G151" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H151" s="15" t="inlineStr">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="G152" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H152" s="15" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="G153" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H153" s="15" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="G154" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H154" s="15" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="G155" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H155" s="15" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="G156" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H156" s="15" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G157" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H157" s="15" t="inlineStr">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G158" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H158" s="15" t="inlineStr">
@@ -7251,7 +7251,7 @@
       </c>
       <c r="G159" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H159" s="15" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="G160" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H160" s="15" t="inlineStr">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="G161" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H161" s="15" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="G162" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H162" s="15" t="inlineStr">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="G163" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H163" s="15" t="inlineStr">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="G164" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H164" s="15" t="inlineStr">
@@ -7487,11 +7487,11 @@
         </is>
       </c>
       <c r="F165" s="17" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G165" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H165" s="15" t="inlineStr">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="G166" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H166" s="15" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="G167" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H167" s="15" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G168" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H168" s="15" t="inlineStr">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="G169" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H169" s="15" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="G170" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H170" s="15" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="G171" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H171" s="15" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="G172" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H172" s="15" t="inlineStr">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="G173" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H173" s="15" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="G174" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H174" s="15" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H175" s="15" t="inlineStr">
@@ -7931,7 +7931,7 @@
       </c>
       <c r="G176" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H176" s="15" t="inlineStr">
@@ -7971,7 +7971,7 @@
       </c>
       <c r="G177" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H177" s="15" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G178" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H178" s="15" t="inlineStr">
@@ -8051,7 +8051,7 @@
       </c>
       <c r="G179" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H179" s="15" t="inlineStr">
@@ -8091,7 +8091,7 @@
       </c>
       <c r="G180" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H180" s="15" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="G181" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H181" s="15" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="G182" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H182" s="15" t="inlineStr">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="G183" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H183" s="15" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="G184" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H184" s="15" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="G185" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H185" s="15" t="inlineStr">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="G186" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H186" s="15" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="G187" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H187" s="15" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="G188" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H188" s="15" t="inlineStr">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="G189" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H189" s="15" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="G190" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H190" s="15" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="G191" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H191" s="15" t="inlineStr">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="G192" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H192" s="15" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="G193" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H193" s="15" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="G194" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H194" s="15" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G195" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H195" s="15" t="inlineStr">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="G196" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H196" s="15" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="G197" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H197" s="15" t="inlineStr">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G198" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H198" s="15" t="inlineStr">
@@ -8851,7 +8851,7 @@
       </c>
       <c r="G199" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H199" s="15" t="inlineStr">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="G200" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H200" s="15" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="G201" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H201" s="15" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="G202" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H202" s="15" t="inlineStr">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G203" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H203" s="15" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="G204" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H204" s="15" t="inlineStr">
@@ -9091,7 +9091,7 @@
       </c>
       <c r="G205" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H205" s="15" t="inlineStr">
@@ -9131,7 +9131,7 @@
       </c>
       <c r="G206" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H206" s="15" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="G207" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H207" s="15" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G208" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H208" s="15" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="G209" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H209" s="15" t="inlineStr">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="G210" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H210" s="15" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="G211" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H211" s="15" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="G212" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H212" s="15" t="inlineStr">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="G213" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H213" s="15" t="inlineStr">
@@ -9451,7 +9451,7 @@
       </c>
       <c r="G214" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H214" s="15" t="inlineStr">
@@ -9491,7 +9491,7 @@
       </c>
       <c r="G215" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H215" s="15" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="G216" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H216" s="15" t="inlineStr">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="G217" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H217" s="15" t="inlineStr">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G218" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H218" s="15" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="G219" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H219" s="15" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="G220" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H220" s="15" t="inlineStr">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="G221" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H221" s="15" t="inlineStr">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="G222" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H222" s="15" t="inlineStr">
@@ -9811,7 +9811,7 @@
       </c>
       <c r="G223" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H223" s="15" t="inlineStr">
@@ -9851,7 +9851,7 @@
       </c>
       <c r="G224" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H224" s="15" t="inlineStr">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="G225" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H225" s="15" t="inlineStr">
@@ -9931,7 +9931,7 @@
       </c>
       <c r="G226" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H226" s="15" t="inlineStr">
@@ -9971,7 +9971,7 @@
       </c>
       <c r="G227" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H227" s="15" t="inlineStr">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="G228" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H228" s="15" t="inlineStr">
@@ -10051,7 +10051,7 @@
       </c>
       <c r="G229" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H229" s="15" t="inlineStr">
@@ -10091,7 +10091,7 @@
       </c>
       <c r="G230" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H230" s="15" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="G231" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H231" s="15" t="inlineStr">
@@ -10171,7 +10171,7 @@
       </c>
       <c r="G232" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H232" s="15" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="G233" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H233" s="15" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="G234" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H234" s="15" t="inlineStr">
@@ -10291,7 +10291,7 @@
       </c>
       <c r="G235" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H235" s="15" t="inlineStr">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="G236" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H236" s="15" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="G237" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H237" s="15" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="G238" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H238" s="15" t="inlineStr">
@@ -10451,7 +10451,7 @@
       </c>
       <c r="G239" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H239" s="15" t="inlineStr">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="G240" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H240" s="15" t="inlineStr">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="G241" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H241" s="15" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="G242" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H242" s="15" t="inlineStr">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="G243" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H243" s="15" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="G244" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H244" s="15" t="inlineStr">
@@ -10691,7 +10691,7 @@
       </c>
       <c r="G245" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H245" s="15" t="inlineStr">
@@ -10731,7 +10731,7 @@
       </c>
       <c r="G246" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H246" s="15" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="G247" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H247" s="15" t="inlineStr">
@@ -10811,7 +10811,7 @@
       </c>
       <c r="G248" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H248" s="15" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="G249" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H249" s="15" t="inlineStr">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="G250" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H250" s="15" t="inlineStr">
@@ -10931,7 +10931,7 @@
       </c>
       <c r="G251" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H251" s="15" t="inlineStr">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="G252" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H252" s="15" t="inlineStr">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="G253" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H253" s="15" t="inlineStr">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="G254" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H254" s="15" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="G255" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H255" s="15" t="inlineStr">
@@ -11131,7 +11131,7 @@
       </c>
       <c r="G256" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H256" s="15" t="inlineStr">
@@ -11171,7 +11171,7 @@
       </c>
       <c r="G257" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H257" s="15" t="inlineStr">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="G258" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H258" s="15" t="inlineStr">
@@ -11251,7 +11251,7 @@
       </c>
       <c r="G259" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H259" s="15" t="inlineStr">
@@ -11291,7 +11291,7 @@
       </c>
       <c r="G260" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H260" s="15" t="inlineStr">
@@ -11331,7 +11331,7 @@
       </c>
       <c r="G261" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H261" s="15" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="G262" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H262" s="15" t="inlineStr">
@@ -11407,11 +11407,11 @@
         </is>
       </c>
       <c r="F263" s="17" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G263" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H263" s="15" t="inlineStr">
@@ -11451,7 +11451,7 @@
       </c>
       <c r="G264" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H264" s="15" t="inlineStr">
@@ -11491,7 +11491,7 @@
       </c>
       <c r="G265" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H265" s="15" t="inlineStr">
@@ -11531,7 +11531,7 @@
       </c>
       <c r="G266" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H266" s="15" t="inlineStr">
@@ -11571,7 +11571,7 @@
       </c>
       <c r="G267" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H267" s="15" t="inlineStr">
@@ -11611,7 +11611,7 @@
       </c>
       <c r="G268" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H268" s="15" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="G269" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H269" s="15" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="G270" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H270" s="15" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="G271" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H271" s="15" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="G272" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H272" s="15" t="inlineStr">
@@ -11811,7 +11811,7 @@
       </c>
       <c r="G273" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H273" s="15" t="inlineStr">
@@ -11851,7 +11851,7 @@
       </c>
       <c r="G274" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H274" s="15" t="inlineStr">
@@ -11891,7 +11891,7 @@
       </c>
       <c r="G275" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H275" s="15" t="inlineStr">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="G276" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H276" s="15" t="inlineStr">
@@ -11971,7 +11971,7 @@
       </c>
       <c r="G277" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H277" s="15" t="inlineStr">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="G278" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H278" s="15" t="inlineStr">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="G279" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H279" s="15" t="inlineStr">
@@ -12091,7 +12091,7 @@
       </c>
       <c r="G280" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H280" s="15" t="inlineStr">
@@ -12131,7 +12131,7 @@
       </c>
       <c r="G281" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H281" s="15" t="inlineStr">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="G282" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H282" s="15" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="G283" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H283" s="15" t="inlineStr">
@@ -12251,7 +12251,7 @@
       </c>
       <c r="G284" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H284" s="15" t="inlineStr">
@@ -12287,11 +12287,11 @@
         </is>
       </c>
       <c r="F285" s="17" t="n">
-        <v>0</v>
+        <v>0.0008</v>
       </c>
       <c r="G285" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H285" s="15" t="inlineStr">
@@ -12331,7 +12331,7 @@
       </c>
       <c r="G286" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H286" s="15" t="inlineStr">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="G287" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H287" s="15" t="inlineStr">
@@ -12411,7 +12411,7 @@
       </c>
       <c r="G288" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H288" s="15" t="inlineStr">
@@ -12451,7 +12451,7 @@
       </c>
       <c r="G289" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H289" s="15" t="inlineStr">
@@ -12491,7 +12491,7 @@
       </c>
       <c r="G290" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H290" s="15" t="inlineStr">
@@ -12527,11 +12527,11 @@
         </is>
       </c>
       <c r="F291" s="17" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="G291" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H291" s="15" t="inlineStr">
@@ -12571,7 +12571,7 @@
       </c>
       <c r="G292" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H292" s="15" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="G293" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H293" s="15" t="inlineStr">
@@ -12651,7 +12651,7 @@
       </c>
       <c r="G294" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H294" s="15" t="inlineStr">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="G295" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H295" s="15" t="inlineStr">
@@ -12727,11 +12727,11 @@
         </is>
       </c>
       <c r="F296" s="17" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="G296" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H296" s="15" t="inlineStr">
@@ -12771,7 +12771,7 @@
       </c>
       <c r="G297" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H297" s="15" t="inlineStr">
@@ -12811,7 +12811,7 @@
       </c>
       <c r="G298" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H298" s="15" t="inlineStr">
@@ -12847,11 +12847,11 @@
         </is>
       </c>
       <c r="F299" s="17" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="G299" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H299" s="15" t="inlineStr">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="G300" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H300" s="15" t="inlineStr">
@@ -12931,7 +12931,7 @@
       </c>
       <c r="G301" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 09:25:00</t>
+          <t>2026-08-07 11:10:39</t>
         </is>
       </c>
       <c r="H301" s="15" t="inlineStr">

</xml_diff>